<commit_message>
feat: verify rule CG0069 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000034/negative/01/data/unit-test-coreid-CG0069-negative.xlsx
+++ b/rules/CORE-000034/negative/01/data/unit-test-coreid-CG0069-negative.xlsx
@@ -613,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -645,6 +645,253 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ds.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DSDECOD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>DEATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ds.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DSSTDTC</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2022-02-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DTHDTC</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2021-02-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ds.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DSDECOD</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DEATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ds.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DSSTDTC</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2019-01-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DTHDTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ds.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DSDECOD</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>DEATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ds.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DSSTDTC</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2021-01-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DTHDTC</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2021-01</t>
         </is>
       </c>
     </row>
@@ -713,7 +960,7 @@
           <t>RFPENDTC</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>DTHDTC</t>
         </is>
@@ -2226,7 +2473,7 @@
           <t>DS</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>015246-076-0003-00003</t>
         </is>
@@ -2847,7 +3094,7 @@
           <t>DS</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>015246-888-0008-08888</t>
         </is>
@@ -3072,7 +3319,7 @@
           <t>DS</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>015246-999-0003-09999</t>
         </is>

</xml_diff>